<commit_message>
Updated excel list and fixed word list for both games
</commit_message>
<xml_diff>
--- a/public/assets/UpdatedAccountingElements.xlsx
+++ b/public/assets/UpdatedAccountingElements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benso\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40557E7F-9BE8-44AF-B817-C76B7734FC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE13A0BA-2020-47C2-8B50-D5A46CE294E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{922BA294-4DCC-45B5-8780-647AD84B5699}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="5" activeTab="8" xr2:uid="{922BA294-4DCC-45B5-8780-647AD84B5699}"/>
   </bookViews>
   <sheets>
     <sheet name="All" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,13 @@
     <sheet name="IS Easy" sheetId="10" r:id="rId6"/>
     <sheet name="IS Medium" sheetId="11" r:id="rId7"/>
     <sheet name="IS Hard" sheetId="12" r:id="rId8"/>
-    <sheet name="Normal Balance Easy" sheetId="14" r:id="rId9"/>
-    <sheet name="Normal Balance Medium" sheetId="15" r:id="rId10"/>
-    <sheet name="Normal Balance Hard" sheetId="16" r:id="rId11"/>
-    <sheet name="A=L+SE - Easy" sheetId="18" r:id="rId12"/>
-    <sheet name="A=L+SE - Medium" sheetId="19" r:id="rId13"/>
-    <sheet name="A=L+SE - Hard" sheetId="20" r:id="rId14"/>
+    <sheet name="Normal Balance - All" sheetId="21" r:id="rId9"/>
+    <sheet name="Normal Balance Easy" sheetId="14" r:id="rId10"/>
+    <sheet name="Normal Balance Medium" sheetId="15" r:id="rId11"/>
+    <sheet name="Normal Balance Hard" sheetId="16" r:id="rId12"/>
+    <sheet name="A=L+SE - Easy" sheetId="18" r:id="rId13"/>
+    <sheet name="A=L+SE - Medium" sheetId="19" r:id="rId14"/>
+    <sheet name="A=L+SE - Hard" sheetId="20" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">All!$A$1:$E$43</definedName>
@@ -37,9 +38,9 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'IS Easy'!$A$1:$B$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'IS Hard'!$A$1:$B$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'IS Medium'!$A$1:$B$43</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Normal Balance Easy'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'Normal Balance Hard'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Normal Balance Medium'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Normal Balance Easy'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'Normal Balance Hard'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'Normal Balance Medium'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1387" uniqueCount="383">
   <si>
     <t>Assets</t>
   </si>
@@ -1667,7 +1668,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E69"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.7109375" bestFit="1" customWidth="1"/>
@@ -2478,12 +2479,408 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F154D7F3-C3D8-4B03-BC6F-5936219A4F16}">
+  <sheetPr codeName="Sheet9">
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B57"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:B31">
+    <sortCondition ref="B2:B31"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="59" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8444ABC8-3E90-4153-947D-671A731C5AD5}">
   <sheetPr codeName="Sheet10">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B76"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42.140625" customWidth="1"/>
@@ -3073,13 +3470,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3178FF7-7A1D-4E9E-B7E2-EC0FF2ACE046}">
   <sheetPr codeName="Sheet11">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B73"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58.140625" bestFit="1" customWidth="1"/>
@@ -3666,10 +4063,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21BE0DBB-C999-5A44-8548-4898BD2D14AB}">
   <dimension ref="B3:F23"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C3" s="5" t="s">
@@ -4027,10 +4424,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{683674F0-791E-8B43-805E-7A46EA7231CA}">
   <dimension ref="B2:G23"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="87.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -4409,12 +4806,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{191C79E7-2766-A64A-8DC8-E055CFAB5B32}">
   <dimension ref="B2:G23"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="92.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="92.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
@@ -4859,7 +5256,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E69"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.42578125" bestFit="1" customWidth="1"/>
@@ -5892,7 +6289,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.7109375" bestFit="1" customWidth="1"/>
@@ -6123,7 +6520,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C39"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.7109375" bestFit="1" customWidth="1"/>
@@ -6472,7 +6869,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.7109375" bestFit="1" customWidth="1"/>
@@ -6818,7 +7215,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
@@ -6997,7 +7394,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B43"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
@@ -7278,7 +7675,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B39"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
@@ -7549,15 +7946,12 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F154D7F3-C3D8-4B03-BC6F-5936219A4F16}">
-  <sheetPr codeName="Sheet9">
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:B57"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1924A69-9EA0-4A41-BBB2-9FB56813B04B}">
+  <dimension ref="A1:B127"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -7804,143 +8198,675 @@
       <c r="A31" s="3" t="s">
         <v>86</v>
       </c>
+      <c r="B31" s="2" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B38" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
         <v>202</v>
       </c>
+      <c r="B56" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:B31">
-    <sortCondition ref="B2:B31"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="59" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8204,16 +9130,16 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75253D14-554A-4916-839F-E7F866211CA3}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="47b4e388-7a75-40af-8b04-42818f2fdb9b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c997e9c3-07ef-4103-ac9e-c49d1d746bce"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c997e9c3-07ef-4103-ac9e-c49d1d746bce"/>
-    <ds:schemaRef ds:uri="47b4e388-7a75-40af-8b04-42818f2fdb9b"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>